<commit_message>
Fix some formatting errors.
</commit_message>
<xml_diff>
--- a/mortality/data_processing_elements_mortality-BCS.xlsx
+++ b/mortality/data_processing_elements_mortality-BCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF62F69A-CCB3-4868-A467-138A392F7B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{71265554-09E7-4594-B192-9DAA27049213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,28 +16,19 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AD$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AB$11</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="95">
-  <si>
-    <t>old_index</t>
-  </si>
-  <si>
-    <t>mid_index</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="93">
   <si>
     <t>index</t>
   </si>
   <si>
     <t>input_dataset</t>
-  </si>
-  <si>
-    <t>name</t>
   </si>
   <si>
     <t>label</t>
@@ -317,6 +308,9 @@
   </si>
   <si>
     <t>Check in user guide if have month.</t>
+  </si>
+  <si>
+    <t>dataschema_variable</t>
   </si>
 </sst>
 </file>
@@ -391,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -414,20 +408,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -763,41 +751,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BO11"/>
+  <dimension ref="A1:BM11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="11.7109375" style="8" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="3.7109375" style="8" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.5703125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="31.140625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="32.28515625" style="8" customWidth="1"/>
-    <col min="8" max="8" width="7.140625" style="8" customWidth="1"/>
-    <col min="9" max="11" width="6" style="8" customWidth="1"/>
-    <col min="12" max="12" width="28.85546875" style="8" customWidth="1"/>
-    <col min="13" max="13" width="21.5703125" style="8" customWidth="1"/>
-    <col min="14" max="14" width="22.85546875" style="9" customWidth="1"/>
-    <col min="15" max="15" width="17.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="27" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.5703125" style="10" customWidth="1"/>
-    <col min="18" max="18" width="7.140625" style="8" customWidth="1"/>
-    <col min="19" max="19" width="24.42578125" style="8" customWidth="1"/>
-    <col min="20" max="20" width="11.85546875" style="8" customWidth="1"/>
-    <col min="21" max="21" width="12.140625" style="8" customWidth="1"/>
-    <col min="22" max="22" width="15" style="8" customWidth="1"/>
-    <col min="23" max="23" width="34.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="20" style="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="31.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21.85546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="31.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="27.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="16.140625" style="8" customWidth="1"/>
-    <col min="30" max="30" width="14.28515625" style="8" customWidth="1"/>
-    <col min="31" max="31" width="9" style="8" customWidth="1"/>
-    <col min="32" max="16384" width="9" style="8"/>
+    <col min="1" max="1" width="3.7109375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="32.28515625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="7.140625" style="8" customWidth="1"/>
+    <col min="7" max="9" width="6" style="8" customWidth="1"/>
+    <col min="10" max="10" width="28.85546875" style="8" customWidth="1"/>
+    <col min="11" max="11" width="21.5703125" style="8" customWidth="1"/>
+    <col min="12" max="12" width="22.85546875" style="9" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="28.5703125" style="10" customWidth="1"/>
+    <col min="16" max="16" width="7.140625" style="8" customWidth="1"/>
+    <col min="17" max="17" width="24.42578125" style="8" customWidth="1"/>
+    <col min="18" max="18" width="11.85546875" style="8" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" style="8" customWidth="1"/>
+    <col min="20" max="20" width="15" style="8" customWidth="1"/>
+    <col min="21" max="21" width="34.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20" style="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="31.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.85546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="27.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.140625" style="8" customWidth="1"/>
+    <col min="28" max="28" width="14.28515625" style="8" customWidth="1"/>
+    <col min="29" max="29" width="9" style="8" customWidth="1"/>
+    <col min="30" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -805,432 +792,397 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="T1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="W1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="X1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="Y1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Z1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="4" t="s">
+      <c r="AB1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AC1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="AD1" s="4" t="s">
-        <v>29</v>
-      </c>
     </row>
-    <row r="2" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="8">
-        <v>1</v>
-      </c>
-      <c r="C2" s="8">
-        <v>1</v>
+      <c r="B2" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>87</v>
+        <v>28</v>
       </c>
       <c r="E2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="M2" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="O2" s="8"/>
+      <c r="R2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="S2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="T2" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="Q2" s="8"/>
-      <c r="T2" s="8" t="s">
-        <v>37</v>
-      </c>
       <c r="U2" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z2" s="8"/>
+        <v>32</v>
+      </c>
+      <c r="X2" s="8"/>
     </row>
-    <row r="3" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2</v>
       </c>
-      <c r="B3" s="8">
-        <v>2</v>
-      </c>
-      <c r="C3" s="8">
-        <v>2</v>
+      <c r="B3" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>37</v>
       </c>
       <c r="D3" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="8"/>
+      <c r="R3" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S3" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="T3" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="X3" s="8"/>
+    </row>
+    <row r="4" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="O4" s="8"/>
+      <c r="R4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="T4" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="U4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="X4" s="8"/>
+    </row>
+    <row r="5" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="O5" s="8"/>
+      <c r="R5" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S5" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="T5" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="U5" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="X5" s="8"/>
+    </row>
+    <row r="6" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="N6" s="9"/>
+      <c r="O6" s="8"/>
+      <c r="Q6" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="8" t="s">
+      <c r="R6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="T6" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="U6" s="8">
+        <v>2021</v>
+      </c>
+      <c r="X6" s="8"/>
+      <c r="Y6" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="M7" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q3" s="8"/>
-      <c r="T3" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="U3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="V3" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="W3" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="Z3" s="8"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="8"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="S7" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="T7" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="U7" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="X7" s="8"/>
+      <c r="Y7" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z7" s="8" t="s">
+        <v>90</v>
+      </c>
     </row>
-    <row r="4" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
-        <v>2</v>
-      </c>
-      <c r="B4" s="8">
-        <v>3</v>
-      </c>
-      <c r="C4" s="8">
-        <v>3</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="F4" s="8" t="s">
+    <row r="8" spans="1:65" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="L4" s="8" t="s">
+      <c r="L8" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="P8" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="R8" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S8" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="O4" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q4" s="8"/>
-      <c r="T4" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="U4" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="V4" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="W4" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="Z4" s="8"/>
-    </row>
-    <row r="5" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
-        <v>3</v>
-      </c>
-      <c r="B5" s="8">
-        <v>4</v>
-      </c>
-      <c r="C5" s="8">
-        <v>4</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="O5" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q5" s="8"/>
-      <c r="T5" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="U5" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="V5" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="W5" s="8" t="s">
+      <c r="T8" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="U8" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="Z5" s="8"/>
-    </row>
-    <row r="6" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
-        <v>4</v>
-      </c>
-      <c r="B6" s="8">
-        <v>5</v>
-      </c>
-      <c r="C6" s="8">
-        <v>5</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="M6" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="O6" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="8"/>
-      <c r="S6" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="T6" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="U6" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="V6" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="W6" s="8">
-        <v>2021</v>
-      </c>
-      <c r="Z6" s="8"/>
-      <c r="AA6" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="AB6" s="12"/>
-    </row>
-    <row r="7" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="C7" s="8">
-        <v>6</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="O7" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="8"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="U7" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="V7" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="W7" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z7" s="8"/>
-      <c r="AA7" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB7" s="12" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="8" spans="1:67" ht="135" x14ac:dyDescent="0.25">
-      <c r="C8" s="8">
-        <v>7</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="N8" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="O8" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="P8" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q8" s="7" t="s">
+      <c r="W8" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y8" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="R8" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="T8" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="U8" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="V8" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="W8" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="Y8" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="AA8" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="AB8" s="11"/>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="10"/>
+      <c r="AB8" s="10"/>
       <c r="AC8" s="10"/>
       <c r="AD8" s="10"/>
       <c r="AE8" s="10"/>
@@ -1268,44 +1220,43 @@
       <c r="BK8" s="10"/>
       <c r="BL8" s="10"/>
       <c r="BM8" s="10"/>
-      <c r="BN8" s="10"/>
-      <c r="BO8" s="10"/>
     </row>
-    <row r="9" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="C9" s="8">
+    <row r="9" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
         <v>8</v>
       </c>
+      <c r="B9" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>61</v>
+      </c>
       <c r="D9" s="8" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="O9" s="8" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="R9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="S9" s="8" t="s">
+        <v>54</v>
       </c>
       <c r="T9" s="8" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="U9" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="V9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="W9" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y9" s="11"/>
+        <v>53</v>
+      </c>
+      <c r="Y9" s="10"/>
+      <c r="Z9" s="10"/>
       <c r="AA9" s="10"/>
       <c r="AB9" s="10"/>
       <c r="AC9" s="10"/>
@@ -1345,48 +1296,47 @@
       <c r="BK9" s="10"/>
       <c r="BL9" s="10"/>
       <c r="BM9" s="10"/>
-      <c r="BN9" s="10"/>
-      <c r="BO9" s="10"/>
     </row>
-    <row r="10" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="C10" s="8">
+    <row r="10" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
         <v>9</v>
       </c>
+      <c r="B10" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="D10" s="8" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="E10" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M10" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="N10" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="O10" s="8"/>
+      <c r="R10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="T10" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="U10" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="O10" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="P10" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q10" s="8"/>
-      <c r="T10" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="U10" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="V10" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="W10" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="Y10" s="11"/>
+      <c r="Y10" s="10"/>
+      <c r="Z10" s="10"/>
       <c r="AA10" s="10"/>
       <c r="AB10" s="10"/>
       <c r="AC10" s="10"/>
@@ -1426,48 +1376,47 @@
       <c r="BK10" s="10"/>
       <c r="BL10" s="10"/>
       <c r="BM10" s="10"/>
-      <c r="BN10" s="10"/>
-      <c r="BO10" s="10"/>
     </row>
-    <row r="11" spans="1:67" x14ac:dyDescent="0.25">
-      <c r="C11" s="8">
+    <row r="11" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
         <v>10</v>
       </c>
+      <c r="B11" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="D11" s="8" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E11" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="N11" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="O11" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="P11" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="R11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S11" s="8" t="s">
+        <v>35</v>
+      </c>
       <c r="T11" s="8" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="U11" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="V11" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="W11" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="Y11" s="11"/>
+        <v>67</v>
+      </c>
+      <c r="Y11" s="10"/>
+      <c r="Z11" s="10"/>
       <c r="AA11" s="10"/>
       <c r="AB11" s="10"/>
       <c r="AC11" s="10"/>
@@ -1507,13 +1456,11 @@
       <c r="BK11" s="10"/>
       <c r="BL11" s="10"/>
       <c r="BM11" s="10"/>
-      <c r="BN11" s="10"/>
-      <c r="BO11" s="10"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD11" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD11">
-      <sortCondition ref="C1:C11"/>
+  <autoFilter ref="A1:AB11" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AB11">
+      <sortCondition ref="A1:A11"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Change variable names to lowercase
</commit_message>
<xml_diff>
--- a/mortality/data_processing_elements_mortality-BCS.xlsx
+++ b/mortality/data_processing_elements_mortality-BCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{71265554-09E7-4594-B192-9DAA27049213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D091BF0E-1989-4F9A-BA96-66325986FA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="94">
   <si>
     <t>index</t>
   </si>
@@ -200,9 +200,6 @@
     <t>Indicator of whether the participant is deceased</t>
   </si>
   <si>
-    <t>OUTCME11</t>
-  </si>
-  <si>
     <t>Outcome to BCS11 (2021)</t>
   </si>
   <si>
@@ -221,9 +218,6 @@
     <t>Death date - Month</t>
   </si>
   <si>
-    <t>DODMTH</t>
-  </si>
-  <si>
     <t>Consolidated month of death</t>
   </si>
   <si>
@@ -234,9 +228,6 @@
   </si>
   <si>
     <t>Death date - Year</t>
-  </si>
-  <si>
-    <t>DODYR</t>
   </si>
   <si>
     <t>Consolidated year of death</t>
@@ -311,6 +302,18 @@
   </si>
   <si>
     <t>dataschema_variable</t>
+  </si>
+  <si>
+    <t>bcsid</t>
+  </si>
+  <si>
+    <t>outcme11</t>
+  </si>
+  <si>
+    <t>dodmth</t>
+  </si>
+  <si>
+    <t>dodyr</t>
   </si>
 </sst>
 </file>
@@ -752,39 +755,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BM11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" style="8" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" style="8" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="32.28515625" style="8" customWidth="1"/>
-    <col min="6" max="6" width="7.140625" style="8" customWidth="1"/>
+    <col min="1" max="1" width="3.7265625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.7265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.54296875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="31.1796875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="32.26953125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="7.1796875" style="8" customWidth="1"/>
     <col min="7" max="9" width="6" style="8" customWidth="1"/>
-    <col min="10" max="10" width="28.85546875" style="8" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" style="8" customWidth="1"/>
-    <col min="12" max="12" width="22.85546875" style="9" customWidth="1"/>
-    <col min="13" max="13" width="17.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.81640625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="21.54296875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="22.81640625" style="9" customWidth="1"/>
+    <col min="13" max="13" width="17.1796875" style="8" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="27" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="28.5703125" style="10" customWidth="1"/>
-    <col min="16" max="16" width="7.140625" style="8" customWidth="1"/>
-    <col min="17" max="17" width="24.42578125" style="8" customWidth="1"/>
-    <col min="18" max="18" width="11.85546875" style="8" customWidth="1"/>
-    <col min="19" max="19" width="12.140625" style="8" customWidth="1"/>
+    <col min="15" max="15" width="28.54296875" style="10" customWidth="1"/>
+    <col min="16" max="16" width="7.1796875" style="8" customWidth="1"/>
+    <col min="17" max="17" width="24.453125" style="8" customWidth="1"/>
+    <col min="18" max="18" width="11.81640625" style="8" customWidth="1"/>
+    <col min="19" max="19" width="12.1796875" style="8" customWidth="1"/>
     <col min="20" max="20" width="15" style="8" customWidth="1"/>
-    <col min="21" max="21" width="34.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="34.7265625" style="8" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="20" style="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="31.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.85546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="31.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="27.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.140625" style="8" customWidth="1"/>
-    <col min="28" max="28" width="14.28515625" style="8" customWidth="1"/>
+    <col min="23" max="23" width="31.54296875" style="10" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.7265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="27.453125" style="8" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.1796875" style="8" customWidth="1"/>
+    <col min="28" max="28" width="14.26953125" style="8" customWidth="1"/>
     <col min="29" max="29" width="9" style="8" customWidth="1"/>
     <col min="30" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -792,7 +795,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -870,12 +873,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>27</v>
@@ -893,7 +896,7 @@
         <v>31</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>32</v>
+        <v>90</v>
       </c>
       <c r="N2" s="8" t="s">
         <v>33</v>
@@ -913,12 +916,12 @@
       </c>
       <c r="X2" s="8"/>
     </row>
-    <row r="3" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>37</v>
@@ -953,12 +956,12 @@
       </c>
       <c r="X3" s="8"/>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>44</v>
@@ -993,21 +996,21 @@
       </c>
       <c r="X4" s="8"/>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>30</v>
@@ -1026,31 +1029,31 @@
         <v>42</v>
       </c>
       <c r="U5" s="8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="X5" s="8"/>
     </row>
-    <row r="6" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>48</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="K6" s="8" t="s">
         <v>49</v>
@@ -1061,7 +1064,7 @@
       <c r="N6" s="9"/>
       <c r="O6" s="8"/>
       <c r="Q6" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="R6" s="8" t="s">
         <v>34</v>
@@ -1077,30 +1080,30 @@
       </c>
       <c r="X6" s="8"/>
       <c r="Y6" s="10" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D7" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>81</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>48</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="M7" s="8" t="s">
         <v>41</v>
@@ -1122,18 +1125,18 @@
       </c>
       <c r="X7" s="8"/>
       <c r="Y7" s="8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="Z7" s="8" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:65" ht="135" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:65" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>55</v>
@@ -1151,16 +1154,16 @@
         <v>52</v>
       </c>
       <c r="M8" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="N8" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="8" t="s">
+      <c r="O8" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="P8" s="8" t="s">
         <v>59</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="P8" s="8" t="s">
-        <v>60</v>
       </c>
       <c r="R8" s="8" t="s">
         <v>34</v>
@@ -1172,13 +1175,13 @@
         <v>51</v>
       </c>
       <c r="U8" s="8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Z8" s="10"/>
       <c r="AA8" s="10"/>
@@ -1221,21 +1224,21 @@
       <c r="BL8" s="10"/>
       <c r="BM8" s="10"/>
     </row>
-    <row r="9" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>62</v>
-      </c>
       <c r="E9" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>48</v>
@@ -1297,30 +1300,30 @@
       <c r="BL9" s="10"/>
       <c r="BM9" s="10"/>
     </row>
-    <row r="10" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>64</v>
-      </c>
       <c r="E10" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>48</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="O10" s="8"/>
       <c r="R10" s="8" t="s">
@@ -1330,10 +1333,10 @@
         <v>35</v>
       </c>
       <c r="T10" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U10" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Y10" s="10"/>
       <c r="Z10" s="10"/>
@@ -1377,30 +1380,30 @@
       <c r="BL10" s="10"/>
       <c r="BM10" s="10"/>
     </row>
-    <row r="11" spans="1:65" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>48</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="O11" s="8"/>
       <c r="R11" s="8" t="s">
@@ -1410,10 +1413,10 @@
         <v>35</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U11" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Y11" s="10"/>
       <c r="Z11" s="10"/>

</xml_diff>

<commit_message>
Remove death date variables - not available
</commit_message>
<xml_diff>
--- a/mortality/data_processing_elements_mortality-BCS.xlsx
+++ b/mortality/data_processing_elements_mortality-BCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D091BF0E-1989-4F9A-BA96-66325986FA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB8A655-9093-4BD8-B568-A1D8C046F204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="88">
   <si>
     <t>index</t>
   </si>
@@ -119,9 +119,6 @@
   </si>
   <si>
     <t>Must be unique within the study.</t>
-  </si>
-  <si>
-    <t>BCSID</t>
   </si>
   <si>
     <t>research case identifier</t>
@@ -218,19 +215,10 @@
     <t>Death date - Month</t>
   </si>
   <si>
-    <t>Consolidated month of death</t>
-  </si>
-  <si>
-    <t>direct_mapping</t>
-  </si>
-  <si>
     <t>dth_date_year</t>
   </si>
   <si>
     <t>Death date - Year</t>
-  </si>
-  <si>
-    <t>Consolidated year of death</t>
   </si>
   <si>
     <t>To help us with the consolidation script, can you verify the format of dataset (file extension).</t>
@@ -308,12 +296,6 @@
   </si>
   <si>
     <t>outcme11</t>
-  </si>
-  <si>
-    <t>dodmth</t>
-  </si>
-  <si>
-    <t>dodyr</t>
   </si>
 </sst>
 </file>
@@ -795,7 +777,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>2</v>
@@ -878,7 +860,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>27</v>
@@ -896,23 +878,23 @@
         <v>31</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O2" s="8"/>
       <c r="R2" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="S2" s="8" t="s">
+      <c r="T2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="T2" s="8" t="s">
-        <v>36</v>
-      </c>
       <c r="U2" s="8" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="X2" s="8"/>
     </row>
@@ -921,38 +903,38 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C3" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>39</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>30</v>
       </c>
       <c r="J3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="O3" s="8"/>
       <c r="R3" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="S3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="S3" s="8" t="s">
-        <v>35</v>
-      </c>
       <c r="T3" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="U3" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="U3" s="8" t="s">
-        <v>43</v>
       </c>
       <c r="X3" s="8"/>
     </row>
@@ -961,38 +943,38 @@
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>45</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>46</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>30</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O4" s="8"/>
       <c r="R4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="S4" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="S4" s="8" t="s">
-        <v>35</v>
-      </c>
       <c r="T4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="U4" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="U4" s="8" t="s">
-        <v>43</v>
       </c>
       <c r="X4" s="8"/>
     </row>
@@ -1001,35 +983,35 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>30</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O5" s="8"/>
       <c r="R5" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="S5" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="S5" s="8" t="s">
-        <v>35</v>
-      </c>
       <c r="T5" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="U5" s="8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="X5" s="8"/>
     </row>
@@ -1038,49 +1020,49 @@
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>77</v>
-      </c>
       <c r="F6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>49</v>
-      </c>
       <c r="M6" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N6" s="9"/>
       <c r="O6" s="8"/>
       <c r="Q6" s="9" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="R6" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="S6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="S6" s="8" t="s">
-        <v>35</v>
-      </c>
       <c r="T6" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="U6" s="8">
         <v>2021</v>
       </c>
       <c r="X6" s="8"/>
       <c r="Y6" s="10" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:65" x14ac:dyDescent="0.35">
@@ -1088,47 +1070,47 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="F7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J7" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>79</v>
-      </c>
       <c r="M7" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="N7" s="9"/>
       <c r="O7" s="8"/>
       <c r="Q7" s="9"/>
       <c r="R7" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="S7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="S7" s="8" t="s">
-        <v>54</v>
-      </c>
       <c r="T7" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="U7" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="X7" s="8"/>
       <c r="Y7" s="8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="Z7" s="8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:65" ht="130.5" x14ac:dyDescent="0.35">
@@ -1136,52 +1118,52 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P8" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="R8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="S8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="T8" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="U8" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="W8" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y8" s="10" t="s">
         <v>81</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="L8" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="M8" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="N8" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="P8" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="R8" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="S8" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="T8" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="U8" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="W8" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="Y8" s="10" t="s">
-        <v>85</v>
       </c>
       <c r="Z8" s="10"/>
       <c r="AA8" s="10"/>
@@ -1229,34 +1211,34 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>61</v>
-      </c>
       <c r="E9" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M9" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="R9" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="S9" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="S9" s="8" t="s">
-        <v>54</v>
-      </c>
       <c r="T9" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="U9" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="Y9" s="10"/>
       <c r="Z9" s="10"/>
@@ -1305,38 +1287,35 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>63</v>
-      </c>
       <c r="E10" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="N10" s="8" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="O10" s="8"/>
       <c r="R10" s="8" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="S10" s="8" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="T10" s="8" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="U10" s="8" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="Y10" s="10"/>
       <c r="Z10" s="10"/>
@@ -1385,38 +1364,35 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="N11" s="8" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="O11" s="8"/>
       <c r="R11" s="8" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="S11" s="8" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="U11" s="8" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="Y11" s="10"/>
       <c r="Z11" s="10"/>

</xml_diff>